<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-07 Le train de Sarah
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-07.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-07.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>maison, après-midi de vent</t>
+          <t>maison, après-midi de vent, salon, jardin, balançoire, porte, vitre, rail, train, wagon, gare du salon</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Sarah, papa</t>
+          <t>Sarah, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Le vent est trop fort pour la balançoire. Sarah dit qu'elle est déçue. Ils font un train en bois. Le wagon rouge manque. Elle prend le bleu.</t>
+          <t>La vitre du salon vibre sous le vent. Sur le bois, un éclat de rail luit. Sarah veut la balançoire, maintenant. Le vent est trop fort. Sourire parti. Poitrine trop pleine. Papa s'accroupit. Je suis déçue. Merci vécu. Un train en bois, alors. Deuxième ruse : le wagon rouge manque. Elle refuse de foncer. Elle prend le bleu. Un éclat de rail tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une chaussette rouge vole au vent. Elle danse sur le fil. Le volet tape une fois, puis encore. La cheminée fait un bruit creux. Les branches frottent la vitre. Ça fait un grattement doux. Le tapis du salon sent le bois. Tu as entendu le volet, Sarah ? Il tape. C'est le vent. Il est très fort, aujourd'hui. En ce moment, Sarah veut le jardin. La balançoire, papa. On regarde par la porte. La balançoire va toute seule. Les chaînes tintent. Le vent est trop fort. Sarah sent ses épaules tomber. Sa gorge se serre. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Sarah souffle une fois. Ses cheveux bougent un peu. Un train en bois, alors. Une autre idée. Bravo, Sarah. Ils posent les rails. Le bois est lisse et clair. Les rails font un petit clic. Tu veux le premier wagon ? Le rouge. Sarah cherche dans la boîte. Il n'y a plus de rouge. Il n'est plus là. Sarah sent encore sa gorge. Je suis déçue. Encore un souhait qui attend. Une autre idée ? Sarah regarde un wagon bleu. Le bleu, alors. Oui. Tu as proposé autre chose. Papa tend le wagon bleu. Sarah le pose sur le rail. Le bois glisse, tout doux. Il avance. Être déçue n'est pas honteux. Une autre idée peut venir. Le volet tape plus loin, plus faible. Le train bleu va jusqu'au bout.</t>
+          <t>La vitre du salon vibre sous le vent. Elle tremble, papa. Tu l'entends, la vitre ? Oui, papa. Sarah connaît cette maison, ses bruits d'après-midi. Tu la connais, cette pièce ? Oui, maman. Un rail de bois attend près de la porte. Il est nouveau. Tu le vois, le rail ? Oui, papa. Sur le bois, un éclat de rail luit. Il brille, maman. Tu le vois, le petit point ? Oui, un point clair. Le vent le touche. Le volet tape une fois contre le mur. Il tape fort. Tu l'entends, le volet ? Oui, maman. La porte laisse passer un souffle froid. Ça sent le dehors. Tu le sens, le vent ? Oui, papa. Sarah pose la main sur la poignée. Elle est froide. Tes doigts sont froids, Sarah ? Un peu, maman. Par la porte, le jardin bouge. Les branches bougent. Tu vois le jardin ? Oui, papa. En ce moment, Sarah veut le jardin. La balançoire, maintenant ! Tout de suite ? Oui, papa. Sarah pousse la porte trop vite. Le vent entre d'un coup. Il pousse ! On regarde par la porte ? Oui, maman. La balançoire va toute seule, dans le jardin. Elle part sans moi. Les chaînes tintent, Sarah ? Oui, fort. Le vent est trop fort, près des chaînes. Je veux y aller. Sarah avance un pied dehors, trop vite. Le vent lui rentre dans les cheveux. Ça pique les yeux. Tu recules, Sarah ? Un peu. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Sarah ? Un peu, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Sarah ? Un peu, maman. Je suis déçue. L'éclat de rail tremble, puis tient. Tu vois le jardin, Sarah ? Oui. Sarah serre les poings, puis les ouvre. Tes poings, Sarah ? Ils se desserrent.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une chaussette rouge vole au vent. Elle danse sur le fil. Le volet tape une fois, puis encore. La cheminée fait un bruit creux. Les branches frottent la vitre. Ça fait un grattement doux. Le tapis du salon sent le bois. Tu as entendu le volet, Sarah ? Il tape. C'est le vent. Il est très fort, aujourd'hui. En ce moment, Sarah veut le jardin. La balançoire, papa. On regarde par la porte. La balançoire va toute seule. Les chaînes tintent. Le vent est trop fort. Sarah sent ses épaules tomber. Sa gorge se serre. Je suis déçue. Tu es déçue. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Sarah souffle une fois. Ses cheveux bougent un peu. Un train en bois, alors. Une autre idée. Bravo, Sarah. Ils posent les rails. Le bois est lisse et clair. Les rails font un petit clic. Tu veux le premier wagon ? Le rouge. Sarah cherche dans la boîte. Il n'y a plus de rouge. Il n'est plus là. Sarah sent encore sa gorge. Je suis déçue. Encore un souhait qui attend. Une autre idée ? Sarah regarde un wagon bleu. Le bleu, alors. Oui. Tu as proposé autre chose. Papa tend le wagon bleu. Sarah le pose sur le rail. Le bois glisse, tout doux. Il avance. Être déçue n'est pas honteux. Une autre idée peut venir. Le volet tape plus loin, plus faible. Le train bleu va jusqu'au bout.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;La vitre du salon vibre sous le vent. Elle tremble, papa. Tu l'entends, la vitre ? Oui, papa. Sarah connaît cette maison, ses bruits d'après-midi. Tu la connais, cette pièce ? Oui, maman. Un rail de bois attend près de la porte. Il est nouveau. Tu le vois, le rail ? Oui, papa. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de rail&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un point clair. Le vent le touche. Le volet tape une fois contre le mur. Il tape fort. Tu l'entends, le volet ? Oui, maman. La porte laisse passer un souffle froid. Ça sent le dehors. Tu le sens, le vent ? Oui, papa. Sarah pose la main sur la poignée. Elle est froide. Tes doigts sont froids, Sarah ? Un peu, maman. Par la porte, le jardin bouge. Les branches bougent. Tu vois le jardin ? Oui, papa. En ce moment, Sarah veut le jardin. La balançoire, maintenant ! Tout de suite ? Oui, papa. Sarah pousse la porte trop vite. Le vent entre d'un coup. Il pousse ! On regarde par la porte ? Oui, maman. La balançoire va toute seule, dans le jardin. Elle part sans moi. Les chaînes tintent, Sarah ? Oui, fort. Le vent est trop fort, près des chaînes. Je veux y aller. Sarah avance un pied dehors, trop vite. Le vent lui rentre dans les cheveux. Ça pique les yeux. Tu recules, Sarah ? Un peu. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Sarah ? Un peu, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Sarah ? Un peu, maman. Je suis déçue. L'éclat de rail tremble, puis tient. Tu vois le jardin, Sarah ? Oui. Sarah serre les poings, puis les ouvre. Tes poings, Sarah ? Ils se desserrent.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Gaëtane veut la balançoire du jardin. Le vent est trop fort. Les branches tapent. Gaëtane sent ses épaules tomber. Sa gorge se serre. Gaëtane dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Papa s'accroupit. Papa dit : un souhait peut attendre. On peut chercher une autre idée. Gaëtane souffle. Elle dit : on peut faire un train en bois. Papa sourit. Ils posent les rails. Le bois est lisse. Plus tard, Gaëtane veut le wagon rouge. Il n'est plus dans la boîte. Gaëtane sent encore sa gorge. Elle dit : je suis déçue. Puis elle cherche une autre idée. Elle dit : le wagon bleu, alors. Papa le tend. Être déçu n'est pas honteux. Une autre idée peut venir. [pause]</t>
+          <t>La vitre du salon vibre sous le vent. Elle tremble, papa. Tu l'entends, la vitre ? Oui, papa. Sarah connaît cette maison, ses bruits d'après-midi. Tu la connais, cette pièce ? Oui, maman. Un rail de bois attend près de la porte. Il est nouveau. Tu le vois, le rail ? Oui, papa. Sur le bois, un &lt;emphasis&gt;éclat de rail&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, le petit point ? Oui, un point clair. Le vent le touche. Le volet tape une fois contre le mur. Il tape fort. Tu l'entends, le volet ? Oui, maman. La porte laisse passer un souffle froid. Ça sent le dehors. Tu le sens, le vent ? Oui, papa. Sarah pose la main sur la poignée. Elle est froide. Tes doigts sont froids, Sarah ? Un peu, maman. Par la porte, le jardin bouge. Les branches bougent. Tu vois le jardin ? Oui, papa. En ce moment, Sarah veut le jardin. La balançoire, maintenant ! Tout de suite ? Oui, papa. Sarah pousse la porte trop vite. Le vent entre d'un coup. Il pousse ! On regarde par la porte ? Oui, maman. La balançoire va toute seule, dans le jardin. Elle part sans moi. Les chaînes tintent, Sarah ? Oui, fort. Le vent est trop fort, près des chaînes. Je veux y aller. Sarah avance un pied dehors, trop vite. Le vent lui rentre dans les cheveux. Ça pique les yeux. Tu recules, Sarah ? Un peu. Le sourire de Sarah disparaît. Dans sa poitrine, l'envie et l'inquiétude se bousculent. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Sarah ? Un peu, papa. Papa s'accroupit à la même hauteur. Tes mains sont chaudes, Sarah ? Un peu, maman. Je suis déçue. L'éclat de rail tremble, puis tient. Tu vois le jardin, Sarah ? Oui. Sarah serre les poings, puis les ouvre. Tes poings, Sarah ? Ils se desserrent. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de rail</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,62 +1321,81 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis déception; intensite=2; destinataire=enfant; sous_texte=elle_veut_la_balancoire_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une chaussette rouge vole au vent.
-narrateur|Elle danse sur le fil.
-narrateur|Le volet tape une fois, puis encore.
-narrateur|La cheminée fait un bruit creux.
-narrateur|Les branches frottent la vitre.
-narrateur|Ça fait un grattement doux.
-narrateur|Le tapis du salon sent le bois.
-papa|Tu as entendu le volet, Sarah ?
-enfant-f|Il tape.
-papa|C'est le vent.
-papa|Il est très fort, aujourd'hui.
+          <t>narrateur|La vitre du salon vibre sous le vent.
+enfant-f|Elle tremble, papa.
+papa|Tu l'entends, la vitre ?
+enfant-f|Oui, papa.
+narrateur|Sarah connaît cette maison, ses bruits d'après-midi.
+maman|Tu la connais, cette pièce ?
+enfant-f|Oui, maman.
+narrateur|Un rail de bois attend près de la porte.
+enfant-f|Il est nouveau.
+papa|Tu le vois, le rail ?
+enfant-f|Oui, papa.
+narrateur|Sur le bois, un éclat de rail luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, le petit point ?
+enfant-f|Oui, un point clair.
+papa|Le vent le touche.
+narrateur|Le volet tape une fois contre le mur.
+enfant-f|Il tape fort.
+maman|Tu l'entends, le volet ?
+enfant-f|Oui, maman.
+narrateur|La porte laisse passer un souffle froid.
+enfant-f|Ça sent le dehors.
+papa|Tu le sens, le vent ?
+enfant-f|Oui, papa.
+narrateur|Sarah pose la main sur la poignée.
+enfant-f|Elle est froide.
+maman|Tes doigts sont froids, Sarah ?
+enfant-f|Un peu, maman.
+narrateur|Par la porte, le jardin bouge.
+enfant-f|Les branches bougent.
+papa|Tu vois le jardin ?
+enfant-f|Oui, papa.
 narrateur|En ce moment, Sarah veut le jardin.
-enfant-f|La balançoire, papa.
-papa|On regarde par la porte.
-narrateur|La balançoire va toute seule.
-narrateur|Les chaînes tintent.
-papa|Le vent est trop fort.
-narrateur|Sarah sent ses épaules tomber.
-narrateur|Sa gorge se serre.
+enfant-f|La balançoire, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Sarah pousse la porte trop vite.
+narrateur|Le vent entre d'un coup.
+enfant-f|Il pousse !
+maman|On regarde par la porte ?
+enfant-f|Oui, maman.
+narrateur|La balançoire va toute seule, dans le jardin.
+enfant-f|Elle part sans moi.
+papa|Les chaînes tintent, Sarah ?
+enfant-f|Oui, fort.
+narrateur|Le vent est trop fort, près des chaînes.
+enfant-f|Je veux y aller.
+narrateur|Sarah avance un pied dehors, trop vite.
+narrateur|Le vent lui rentre dans les cheveux.
+enfant-f|Ça pique les yeux.
+maman|Tu recules, Sarah ?
+enfant-f|Un peu.
+narrateur|Le sourire de Sarah disparaît.
+narrateur|Dans sa poitrine, l'envie et l'inquiétude se bousculent.
+narrateur|Ses épaules tombent un peu.
+enfant-f|J'ai mal au ventre.
+papa|Ta gorge est serrée, Sarah ?
+enfant-f|Un peu, papa.
+narrateur|Papa s'accroupit à la même hauteur.
+maman|Tes mains sont chaudes, Sarah ?
+enfant-f|Un peu, maman.
 enfant-f|Je suis déçue.
-papa|Tu es déçue.
-papa|Ce n'est pas honteux.
-papa|Un souhait peut attendre.
-papa|On peut chercher une autre idée.
-narrateur|Sarah souffle une fois.
-narrateur|Ses cheveux bougent un peu.
-enfant-f|Un train en bois, alors.
-papa|Une autre idée.
-papa|Bravo, Sarah.
-narrateur|Ils posent les rails.
-narrateur|Le bois est lisse et clair.
-narrateur|Les rails font un petit clic.
-papa|Tu veux le premier wagon ?
-enfant-f|Le rouge.
-narrateur|Sarah cherche dans la boîte.
-narrateur|Il n'y a plus de rouge.
-papa|Il n'est plus là.
-narrateur|Sarah sent encore sa gorge.
-enfant-f|Je suis déçue.
-papa|Encore un souhait qui attend.
-papa|Une autre idée ?
-narrateur|Sarah regarde un wagon bleu.
-enfant-f|Le bleu, alors.
-papa|Oui.
-papa|Tu as proposé autre chose.
-narrateur|Papa tend le wagon bleu.
-narrateur|Sarah le pose sur le rail.
-narrateur|Le bois glisse, tout doux.
-enfant-f|Il avance.
-papa|Être déçue n'est pas honteux.
-papa|Une autre idée peut venir.
-narrateur|Le volet tape plus loin, plus faible.
-narrateur|Le train bleu va jusqu'au bout.</t>
+narrateur|L'éclat de rail tremble, puis tient.
+papa|Tu vois le jardin, Sarah ?
+enfant-f|Oui.
+narrateur|Sarah serre les poings, puis les ouvre.
+papa|Tes poings, Sarah ?
+enfant-f|Ils se desserrent.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1413,12 +1432,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Le vent est trop fort. Que dit Sarah ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Le vent est trop fort. Que dit &lt;emphasis level="moderate"&gt;Sarah&lt;/emphasis&gt; ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Le vent est trop fort. Que dit Gaëtane ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Le vent est trop fort. Que dit &lt;emphasis&gt;Sarah&lt;/emphasis&gt; ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1443,7 +1462,7 @@
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Gaëtane cherche une autre idée. Que dit-elle d'abord ?</t>
+          <t>Sarah cherche une autre idée. Que dit-elle d'abord ?</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr"/>
@@ -1481,7 +1500,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1492,7 +1511,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1507,34 +1526,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1549,17 +1572,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=le_vent_est_trop_fort_que_dit_sarah; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1592,17 +1615,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Sarah tient encore le wagon bleu. J'ai dit : je suis déçue. Oui. Le souhait peut attendre. Une autre idée est arrivée. Le train, puis le wagon bleu. Bravo, Sarah. Deux autres idées. Oui. Un rail reste tiède sous sa main.</t>
+          <t>Sarah avance un pied vers le jardin, trop vite. J'y vais, maintenant ! Les mots se bousculent dans sa bouche. La balançoire. Sarah avance les mains, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le rail, un instant. Elle écoute la maison, près de la porte. Un train en bois, alors. Tu le vois, le train ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. Le bois du rail est froid, sous les doigts. Il est lisse. Ils posent les rails, sans se presser. Ça fait clic. Tu entends le clic, Sarah ? Oui, papa. Le train tient, Sarah ? Oui, maman. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Jusqu'à la gare du salon. On y va, sans se presser ? Oui. Sarah pose une locomotive, très petite. Elle attend. Tes joues sont chaudes, Sarah ? Un peu, maman. Le premier wagon, plus tard. Oui, papa. Le vent tape plus loin, plus faible. Il est dehors. On reste près des rails ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Sarah tient encore le wagon bleu. J'ai dit : je suis déçue. Oui. Le souhait peut attendre. Une autre idée est arrivée. Le train, puis le wagon bleu. Bravo, Sarah. Deux autres idées. Oui. Un rail reste tiède sous sa main.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah avance un pied vers le jardin, trop vite. J'y vais, maintenant ! Les mots se bousculent dans sa bouche. La balançoire. Sarah avance les mains, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le rail, un instant. Elle écoute la maison, près de la porte. Un &lt;emphasis level="moderate"&gt;train&lt;/emphasis&gt; en bois, alors. Tu le vois, le train ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. Le bois du rail est froid, sous les doigts. Il est lisse. Ils posent les rails, sans se presser. Ça fait clic. Tu entends le clic, Sarah ? Oui, papa. Le train tient, Sarah ? Oui, maman. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Jusqu'à la gare du salon. On y va, sans se presser ? Oui. Sarah pose une locomotive, très petite. Elle attend. Tes joues sont chaudes, Sarah ? Un peu, maman. Le premier wagon, plus tard. Oui, papa. Le vent tape plus loin, plus faible. Il est dehors. On reste près des rails ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Gaëtane a nommé : &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Le souhait peut attendre. Une autre idée est arrivée. Papa était là. [pause]</t>
+          <t>Sarah avance un pied vers le jardin, trop vite. J'y vais, maintenant ! Les mots se bousculent dans sa bouche. La balançoire. Sarah avance les mains, trop vite. Puis elle s'arrête. Sarah refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le rail, un instant. Elle écoute la maison, près de la porte. Un &lt;emphasis&gt;train&lt;/emphasis&gt; en bois, alors. Tu le vois, le train ? Oui, papa. Merci, Sarah. Papa reste à la même hauteur. Le bois du rail est froid, sous les doigts. Il est lisse. Ils posent les rails, sans se presser. Ça fait clic. Tu entends le clic, Sarah ? Oui, papa. Le train tient, Sarah ? Oui, maman. Le ventre de Sarah se desserre. Les épaules se relèvent un peu. Jusqu'à la gare du salon. On y va, sans se presser ? Oui. Sarah pose une locomotive, très petite. Elle attend. Tes joues sont chaudes, Sarah ? Un peu, maman. Le premier wagon, plus tard. Oui, papa. Le vent tape plus loin, plus faible. Il est dehors. On reste près des rails ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1649,7 +1672,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1657,10 +1680,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1683,30 +1706,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>train</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1715,10 +1738,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1731,21 +1754,50 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=elle_prend_le_train_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Sarah tient encore le wagon bleu.
-enfant-f|J'ai dit : je suis déçue.
-papa|Oui.
-papa|Le souhait peut attendre.
-papa|Une autre idée est arrivée.
-papa|Le train, puis le wagon bleu.
-papa|Bravo, Sarah.
-enfant-f|Deux autres idées.
-papa|Oui.
-narrateur|Un rail reste tiède sous sa main.</t>
+          <t>narrateur|Sarah avance un pied vers le jardin, trop vite.
+enfant-f|J'y vais, maintenant !
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|La balançoire.
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Sarah refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le rail, un instant.
+narrateur|Elle écoute la maison, près de la porte.
+enfant-f|Un train en bois, alors.
+papa|Tu le vois, le train ?
+enfant-f|Oui, papa.
+papa|Merci, Sarah.
+narrateur|Papa reste à la même hauteur.
+maman|Le bois du rail est froid, sous les doigts.
+enfant-f|Il est lisse.
+narrateur|Ils posent les rails, sans se presser.
+enfant-f|Ça fait clic.
+papa|Tu entends le clic, Sarah ?
+enfant-f|Oui, papa.
+maman|Le train tient, Sarah ?
+enfant-f|Oui, maman.
+narrateur|Le ventre de Sarah se desserre.
+narrateur|Les épaules se relèvent un peu.
+enfant-f|Jusqu'à la gare du salon.
+papa|On y va, sans se presser ?
+enfant-f|Oui.
+narrateur|Sarah pose une locomotive, très petite.
+enfant-f|Elle attend.
+maman|Tes joues sont chaudes, Sarah ?
+enfant-f|Un peu, maman.
+papa|Le premier wagon, plus tard.
+enfant-f|Oui, papa.
+narrateur|Le vent tape plus loin, plus faible.
+enfant-f|Il est dehors.
+maman|On reste près des rails ?
+enfant-f|Oui, maman.</t>
         </is>
       </c>
     </row>
@@ -1772,17 +1824,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Sarah pousse le wagon bleu. Papa range un rail de trop. On s'assoit un peu ? Oui, papa. Tu as nommé : déçue. Puis tu as cherché. Le bois sent encore le neuf. La chaussette rouge ne vole plus. Le bleu, il avance bien. Oui. Avec l'autre idée.</t>
+          <t>Sarah cherche dans la boîte, trop vite. Le wagon rouge, maintenant ! Sa main trouve du vide. Il n'y en a plus. Le wagon rouge ? Parti. Les épaules de Sarah retombent. Je le prends, tout de suite ! Sarah avance trop vite vers la boîte. La boîte bascule au bord. Elle part ! Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le rail, un instant. Elle écoute la maison, près du train. Sur le bois, un éclat de rail luit. Là, sur le bois. Tu vois le point, Sarah ? Oui, papa. Un wagon bleu attend au fond de la boîte. Le bleu, alors. Tu le vois, le wagon ? Oui, maman. Sarah prend le wagon bleu, sans se presser. Elle le pose sur le rail. Il glisse ! Tu le tiens, Sarah ? Oui, papa. Le wagon penche, presque tombé. Il reste. Il tient, Sarah ? Oui, maman. Ils poussent le train, ensemble. Le train est prêt, Sarah ? Oui, papa. Le wagon bleu avance, un peu de travers. Ça tient. La gare du salon est proche, Sarah ? Oui, maman. Le bleu s'arrête juste avant de tomber. Il a failli partir.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sarah pousse le wagon bleu. Papa range un rail de trop. On s'assoit un peu ? Oui, papa. Tu as nommé : déçue. Puis tu as cherché. Le bois sent encore le neuf. La chaussette rouge ne vole plus. Le bleu, il avance bien. Oui. Avec l'autre idée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Sarah cherche dans la boîte, trop vite. Le wagon rouge, maintenant ! Sa main trouve du vide. Il n'y en a plus. Le wagon rouge ? Parti. Les épaules de Sarah retombent. Je le prends, tout de suite ! Sarah avance trop vite vers la boîte. La boîte bascule au bord. Elle part ! Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le rail, un instant. Elle écoute la maison, près du train. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de rail&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Sarah ? Oui, papa. Un wagon bleu attend au fond de la boîte. Le bleu, alors. Tu le vois, le wagon ? Oui, maman. Sarah prend le wagon bleu, sans se presser. Elle le pose sur le rail. Il glisse ! Tu le tiens, Sarah ? Oui, papa. Le wagon penche, presque tombé. Il reste. Il tient, Sarah ? Oui, maman. Ils poussent le train, ensemble. Le train est prêt, Sarah ? Oui, papa. Le wagon bleu avance, un peu de travers. Ça tient. La gare du salon est proche, Sarah ? Oui, maman. Le bleu s'arrête juste avant de tomber. Il a failli partir.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Gaëtane pousse le wagon bleu. Papa range un rail. Ils s'assoient. [pause]</t>
+          <t>Sarah cherche dans la boîte, trop vite. Le wagon rouge, maintenant ! Sa main trouve du vide. Il n'y en a plus. Le wagon rouge ? Parti. Les épaules de Sarah retombent. Je le prends, tout de suite ! Sarah avance trop vite vers la boîte. La boîte bascule au bord. Elle part ! Sarah avance les mains, trop vite. Puis elle s'arrête net. Sarah refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le rail, un instant. Elle écoute la maison, près du train. Sur le bois, un &lt;emphasis&gt;éclat de rail&lt;/emphasis&gt; luit. Là, sur le bois. Tu vois le point, Sarah ? Oui, papa. Un wagon bleu attend au fond de la boîte. Le bleu, alors. Tu le vois, le wagon ? Oui, maman. Sarah prend le wagon bleu, sans se presser. Elle le pose sur le rail. Il glisse ! Tu le tiens, Sarah ? Oui, papa. Le wagon penche, presque tombé. Il reste. Il tient, Sarah ? Oui, maman. Ils poussent le train, ensemble. Le train est prêt, Sarah ? Oui, papa. Le wagon bleu avance, un peu de travers. Ça tient. La gare du salon est proche, Sarah ? Oui, maman. Le bleu s'arrête juste avant de tomber. Il a failli partir. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1829,7 +1881,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1837,10 +1889,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1861,28 +1913,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rail</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1891,10 +1947,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1905,20 +1961,57 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=wagon_rouge_manque_elle_refuse_de_foncer_prend_le_bleu; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Sarah pousse le wagon bleu.
-narrateur|Papa range un rail de trop.
-papa|On s'assoit un peu ?
+          <t>narrateur|Sarah cherche dans la boîte, trop vite.
+enfant-f|Le wagon rouge, maintenant !
+narrateur|Sa main trouve du vide.
+enfant-f|Il n'y en a plus.
+maman|Le wagon rouge ?
+enfant-f|Parti.
+narrateur|Les épaules de Sarah retombent.
+enfant-f|Je le prends, tout de suite !
+narrateur|Sarah avance trop vite vers la boîte.
+narrateur|La boîte bascule au bord.
+enfant-f|Elle part !
+narrateur|Sarah avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Sarah refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le rail, un instant.
+narrateur|Elle écoute la maison, près du train.
+narrateur|Sur le bois, un éclat de rail luit.
+enfant-f|Là, sur le bois.
+papa|Tu vois le point, Sarah ?
 enfant-f|Oui, papa.
-papa|Tu as nommé : déçue.
-papa|Puis tu as cherché.
-narrateur|Le bois sent encore le neuf.
-narrateur|La chaussette rouge ne vole plus.
-enfant-f|Le bleu, il avance bien.
-papa|Oui.
-papa|Avec l'autre idée.</t>
+narrateur|Un wagon bleu attend au fond de la boîte.
+enfant-f|Le bleu, alors.
+maman|Tu le vois, le wagon ?
+enfant-f|Oui, maman.
+narrateur|Sarah prend le wagon bleu, sans se presser.
+narrateur|Elle le pose sur le rail.
+enfant-f|Il glisse !
+papa|Tu le tiens, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le wagon penche, presque tombé.
+enfant-f|Il reste.
+maman|Il tient, Sarah ?
+enfant-f|Oui, maman.
+narrateur|Ils poussent le train, ensemble.
+papa|Le train est prêt, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le wagon bleu avance, un peu de travers.
+enfant-f|Ça tient.
+maman|La gare du salon est proche, Sarah ?
+enfant-f|Oui, maman.
+narrateur|Le bleu s'arrête juste avant de tomber.
+enfant-f|Il a failli partir.</t>
         </is>
       </c>
     </row>
@@ -1945,17 +2038,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Sarah. Le wagon bleu s'arrête au bout.</t>
+          <t>Ils restent près des rails. Maman essuie un peu de poussière. Le rouge n'était pas là, papa. Tu l'as vu, toi ? Oui, la boîte vide. On est bien, ici. Sarah tapote le wagon bleu du doigt. Il a une petite trace. Tu la vois, la trace ? Oui, maman. Le bleu est resté, Sarah. Oui, avec le train. Ça sent le bois, un peu tiède. Et le vent, maman. Oui, dans l'air. La maison est calme, Sarah ? Oui, papa. Le wagon bleu reste sur le rail. Un éclat de rail tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Sarah. Le wagon bleu s'arrête au bout.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près des rails. Maman essuie un peu de poussière. Le rouge n'était pas là, papa. Tu l'as vu, toi ? Oui, la boîte vide. On est bien, ici. Sarah tapote le wagon bleu du doigt. Il a une petite trace. Tu la vois, la trace ? Oui, maman. Le bleu est resté, Sarah. Oui, avec le train. Ça sent le bois, un peu tiède. Et le vent, maman. Oui, dans l'air. La maison est calme, Sarah ? Oui, papa. Le wagon bleu reste sur le rail. Un &lt;emphasis level="moderate"&gt;éclat de rail&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près des rails. Maman essuie un peu de poussière. Le rouge n'était pas là, papa. Tu l'as vu, toi ? Oui, la boîte vide. On est bien, ici. Sarah tapote le wagon bleu du doigt. Il a une petite trace. Tu la vois, la trace ? Oui, maman. Le bleu est resté, Sarah. Oui, avec le train. Ça sent le bois, un peu tiède. Et le vent, maman. Oui, dans l'air. La maison est calme, Sarah ? Oui, papa. Le wagon bleu reste sur le rail. Un &lt;emphasis&gt;éclat de rail&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2002,7 +2095,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2010,10 +2103,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2022,12 +2115,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2036,17 +2129,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de rail</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2055,11 +2152,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2068,27 +2165,46 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis déçue.
-enfant-f|J'ai trouvé une autre idée.
-papa|Bravo, Sarah.
-narrateur|Le wagon bleu s'arrête au bout.</t>
+          <t>narrateur|Ils restent près des rails.
+narrateur|Maman essuie un peu de poussière.
+enfant-f|Le rouge n'était pas là, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, la boîte vide.
+maman|On est bien, ici.
+narrateur|Sarah tapote le wagon bleu du doigt.
+enfant-f|Il a une petite trace.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le bleu est resté, Sarah.
+enfant-f|Oui, avec le train.
+narrateur|Ça sent le bois, un peu tiède.
+enfant-f|Et le vent, maman.
+maman|Oui, dans l'air.
+papa|La maison est calme, Sarah ?
+enfant-f|Oui, papa.
+narrateur|Le wagon bleu reste sur le rail.
+narrateur|Un éclat de rail tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2225,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2159,6 +2275,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>